<commit_message>
Upgrade crawler with 7 categories, clustering engine, and balanced email layout
</commit_message>
<xml_diff>
--- a/reports/2026-10-13_데일리_이슈_및_금융동향_브리핑.xlsx
+++ b/reports/2026-10-13_데일리_이슈_및_금융동향_브리핑.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="종합이슈_브리핑" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="7대분야_종합이슈" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="주식_환율_경제동향" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="종목분석_매매추천" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
@@ -454,17 +454,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="65" customWidth="1" min="3" max="3"/>
     <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="53" customWidth="1" min="6" max="6"/>
-    <col width="65" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,11 +499,6 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>연결된전일이슈</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>발행일시</t>
         </is>
       </c>
@@ -512,49 +506,44 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>주요사건/사회</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속 보도)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>[속보] 인천 구월동 CGV서 잇단 흉기 난동 신고…부상자 다수 발생</t>
+          <t>여야, 공수처역량 질타…"한동훈 빠져나가"·"김현지 수사 안해"</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>[속보] 인천 구월동 CGV서 잇단 흉기 난동 신고…부상자 다수 발생  뉴스1인천 구월동 흉기난동 1명 심정지·8명 부상 [포토뉴스]  경기일보인천 구월동 홈플러스서 전자발찌 찬 60대 칼부림…1명 심정지·8명 부상(종합)  뉴스1인천 홈플러스 입점 건물서 칼부림…1명 심정지·8명 부상(종합)  뉴시스전자발찌 차고 인천 ...</t>
+          <t>(서울=연합뉴스) 최평천 기자 = 여야는 13일 국회 법제사법위원회의 고위공직자범죄수사처(공수처)에 대한 국정감사에서 공수처의 수사 역량을 질타...</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>뉴스1</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiVEFVX3lxTFByOVhENHZSUURLVVZkQ0pVRmpxWndmQy1zd2N2V1ZobU9mTktkay02bExjSF9vTHFqOWpPeDUtX1pVZXptQ3dMNTZUR0JLUWFsYkt4dw?oc=5</t>
+          <t>https://www.yna.co.kr/view/AKR20261013166400001</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>[속보] 경찰 "홈플러스 인천 구월점 칼부림 부상자 8명…1명 심정지"</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 05:17:39 GMT</t>
+          <t>Tue, 13 Oct 2026 17:26:50 +0900</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>주요사건/사회</t>
+          <t>정치</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -564,92 +553,86 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>특검, ‘대선 허위사실 공표 혐의’ 윤석열 항소심서도 당선무효형 구형</t>
+          <t>"오래된 불발탄도 폭발"…18전투비행단, 고물상 현장 교육</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>특검, ‘대선 허위사실 공표 혐의’ 윤석열 항소심서도 당선무효형 구형  한겨레'국힘 397억 반환' 걸린 尹 재판서 특검 '당선무효형 유지' 요청  MBC 뉴스‘국힘 397억원’ 달린 尹 선거법 2심, 27일 선고  국민일보'선거비용 397억원' 걸린 尹선거법 위반…"항소기각" vs "언어 왜곡" - 머니투데이  머니투데...</t>
+          <t>(강릉=연합뉴스) 유형재 기자 = 공군 제18전투비행단(이하 18전비) 폭발물처리반(이하 EOD)은 최근 3주간 강원 영동지역 민간업체를 대상으...</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>한겨레</t>
+          <t>주요언론</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMickFVX3lxTFBHZ3hUeXlZcERRVkFnUDFtUl9MWjBPWmhaelBmV0VqYU42dnctOW1RMExQcHhFN0dOOXAyX2lFYUtNQnNCX1JVM25OZ1pwZnJZSW9DN19MTGppblZBcDZGV1YtQWdsdGF6T3R4R3JzM1hudw?oc=5</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 05:44:00 GMT</t>
+          <t>https://www.yna.co.kr/view/AKR20261013167200062</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 17:26:35 +0900</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>주요사건/사회</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>연결 이슈 (후속 보도)</t>
+          <t>신규 이슈</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>법무·외교·국방부도 세종 간다…1만명 2031년까지 '대이동'</t>
+          <t>[환율 전망] 대외 악재는 산더미, 반도체 하나로 딸깍</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>법무·외교·국방부도 세종 간다…1만명 2031년까지 '대이동'  한국경제외교부·통일부·국방부... 44개 기관 세종시로 이전  조선일보윤호중 "이전 대상은 총 44개 기관...공무원 9,929명 규모" [현장영상+]  YTN정부 "내년 27개 정부 기관 세종 이전‥금융위·방미통위 등 대상"  MBC 뉴스부산이 원했던 금융...</t>
+          <t>[환율 전망] 대외 악재는 산더미, 반도체 하나로 딸깍  KB Think중동발 유가상승·증시 급락에…환율 10원 오른 1,345.1원  연합뉴스원/달러 환율, 하루 만에 10원 급등…외국인 순매도·달러 강세 - 머니투데이  머니투데이원화값 1330원대 강세…삼성전자 배당·美 금리가 변수...</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>한국경제</t>
+          <t>KB Think</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE5kQk15Qmc2d3RJeEVTWGhHc25SMzFfWENYa191Tk5FZl90ZTUtd1R6Rk95eFFrTU1MRXRSNFNNYXFVbTIxREc3VGp5blpzRkF1Z1hBYTNvQU1NQQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTE9oZVBSLS0wOGtxWUkzN2ZWMEhBVUdROUJiQ3BCNl9QQ2NEemtackZwcVhRZXFOQllTcHJFQWRDdk1sRFZFaFVuX1FMbGZ5Z0E3YV9aOWJIaWJ6TEFCN1B1cQ?oc=5</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>[속보] 외교·통일·국방 등 44개 정부기관, 2031년까지 세종 이전</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 05:10:02 GMT</t>
+          <t>Tue, 13 Oct 2026 08:11:36 GMT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>주요사건/사회</t>
+          <t>거시경제/비즈니스</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>연결 이슈 (후속)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>강경화, 北 지뢰 도발에 "불의의 사고는 분명히 아니다"</t>
+          <t>IMF, 韓 성장률 3.3%로 석 달 만에 0.7%포인트 상향</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>강경화, 北 지뢰 도발에 "불의의 사고는 분명히 아니다"  조선일보강경화 “지뢰, 불의의 사고는 분명히 아니다”… 李대통령 발언 정면반박  문화일보청와대, ‘강경화 불의의 사고 분명 아니다’는 “이 대통령 발언 반박 아냐”  한겨레MDL 넘기가 ‘일과’ 됐나…합참 "지금도 계속되고 있다"  JTBC"왜 도발이라 못하나"·...</t>
+          <t>IMF, 韓 성장률 3.3%로 석 달 만에 0.7%포인트 상향  조선일보[속보]IMF, 한국 올해 성장률 ‘3.3%’까지 올려···석 달 만에 0.7%P 다시 상향  경향신문IMF, 韓성장률 전망치 3.3%로 올렸다…6년만에 세계경제 성장률 넘나 - 머니투데이  머니투데이성장 3%, 소...</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -659,20 +642,19 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMihAFBVV95cUxOVGZTSWRjaEdQRWVzRVBZX3ZNb2UtNkZYeDFRRzdBQmlrLXBFS01waTdKa1lfQl9uTUVfejhHYUpYWGhiNjZwV0F1NmRWZWM1ZTUwSWYzc2JxdFRldVhBOWZ5Z0Y3SE9oYy1ZN091WndvbkVyS0llTmtVVXI5N3pnbjNRTDI?oc=5</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Mon, 12 Oct 2026 19:45:00 GMT</t>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxOX0JSM3hEUGxqOUxodTlWSWl6OGJpRHpIb25uNzNNOXBtdEhmejE5eG1vM3NpWGx3NUJDalhMUDlYdGVkWmFaZThXay1TYjFFaExxdHJqYmlmaEZKa2xCdkk0cUZlRktWZHc5dlo3MlJVOHVGUVlRX25TSHVFU1hoVVYxenBhcEZRUy13akpn?oc=5</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 02:06:05 GMT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>주요사건/사회</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -682,65 +664,71 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>서울 비우고 행정수도 세종으로…일극체제 넘어 균형발전 이룰까</t>
+          <t>러·우·이란·사우디 모두 전쟁… "유럽~아시아 하늘길 역대 가장 위험"</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>(서울=연합뉴스) 양정우 차민지 홍준석 기자 = 정부가 내년부터 시작해 2031년까지 서울과 경기 등 수도권에 소재한 중앙행정기관(부처) 등 4...</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>러·우·이란·사우디 모두 전쟁… "유럽~아시아 하늘길 역대 가장 위험"  조선일보리야드 하늘길 마비·항공편 차질...이란 "대화 중재하겠다"  YTN 사이언스사우디, 방공망·경보발령 '실패' 자체조사 착수(종합)  연합뉴스후티 반군 "美 내전 개입 시 고통스러운 보복" 경고  MBC 뉴...</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>조선일보</t>
+        </is>
+      </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261013147500530</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 16:25:42 +0900</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxNSkJSVFRvcGg0aGlvMjl2YWZ4S0ZOOFVLRlhKVTBrdHpxV2htNWp3Uld6Z0tWWHptMEVCWWpONDFxZGd3czJJVVNkZUcwSzdISTVrNS05UFpkM05aNThVckZ4ZzFITE9hNU50ZHNJU0s0VGxQVlpqRlVuQ3g2MnN4Q1BsQW43SFBkQ1lNdk1Lam1MQ0ZabDZRa2NybTBLZw?oc=5</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Mon, 12 Oct 2026 15:48:00 GMT</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>주요사건/사회</t>
+          <t>세계/국제</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>신규 이슈</t>
+          <t>🔥 [언론사 집중 보도 (5개사)]</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>경기교육청 국감, '교육교부금 개편 찬반' 쟁점 전망</t>
+          <t>트럼프 "중간선거 민주당 이기면 대공황…美 파탄날 것"</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>(수원=연합뉴스) 이영주 기자 = 14일 열리는 국회 교육위원회의 경기도교육청 국정감사에서는 정부의 지방교육재정교부금(교육교부금) 개편을 둘러싸...</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>트럼프 "중간선거 민주당 이기면 대공황…美 파탄날 것"  아시아경제트럼프 "민주당 중간선거 이기면 대공황 온다"  연합인포맥스"트럼프 탓"…텃밭까지 흔들린 공화당, 중간선거 '비상'  마켓인트럼프 경제정책 지지율 25%…중간선거 앞두고 민심 악화  글로벌이코노믹중간 선거 유세서 춤추는 ...</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>아시아경제</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.yna.co.kr/view/AKR20261013142300061</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 16:24:18 +0900</t>
+          <t>https://news.google.com/rss/articles/CBMiYEFVX3lxTFBzcTdtbjZFcG51dGQxTXY3bVp5WFRkbzB2b3FvN2JFeHdILU9OS3otTnp0V3IwbEtNYkJhekZJSVRZcnBEVVJDNGhyeTFOaTZ0LWs5ZHJfTFJpUEpsaTNZNw?oc=5</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 05:20:32 GMT</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>경제/비즈니스</t>
+          <t>연예/대중문화</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -750,264 +738,27 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>윤종군 “기차역 커피·빵 주문 서비스 SPC가 20개월간 독점” 쓴소리</t>
+          <t>영화도 보고 억새축제도 즐기고…합천서 가을 맞아 축제 풍성</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>전국 기차역에서 커피와 빵을 미리 주문할 수 있는 서비스에 SPC 계열업체만 입점해 사실상 독점하고 있다는 주장이 제기됐다. 국회 국토교통위원회 소속 더불어민주당 윤종군 의원(경기..</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>(합천=연합뉴스) 김동민 기자 = 경남 합천군은 가을을 맞아 16일부터 18일까지 제7회 수려한합천영화제를, 17일부터 25일까지 제5회 황매산...</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>주요언론</t>
+        </is>
+      </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>https://www.mk.co.kr/news/economy/12174596</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 16:30:45 +09:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>후티 반군 “美 개입하면 고통스러운 보복” 경고</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>후티 반군 “美 개입하면 고통스러운 보복” 경고  동아일보사우디, 방공망·경보발령 '실패' 자체조사 착수(종합)  연합뉴스브렌트유 한달만에 최고가…국내 기업-소비자 물가 부담 우려  동아일보후티 반군 "美 내전 개입 시 고통스러운 보복" 경고  MBC 뉴스후티發 중동 위기 고조…'딜레마' 빠진 트럼프 美행정부  마켓인</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>동아일보</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTE94UTdzSTFIbXl1TUdiRV92cHllZ25fOTBqRU9YeU5lQ3hTekpfWTFUdEZhZDhPZ3plYnNaalB1VHJnc2Vqd1V6UlgxY2QyZmc3amNPWjB0ekYzQkpSblFxRVNNZkthMjFLWlYxdDZkaFEtb0nSAWZBVV95cUxQMFFZT2NuUjZQcWluZ0laeFFHdjczSFQ5WE9TZnlFVTZTZ3Jzb0RYbW5Gc0gwdnc2LWpuV2E2MU1GNnBPYUJkNWRyTmx6NzhuRTVhY3dMSy1QelFGWC1NMFpKTWpHWXc?oc=5</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 02:47:00 GMT</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속 보도)</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>러, 트럼프 ‘에너지 휴전’ 발표에 “회담 진행 중”…우크라 공격은 지속</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>러, 트럼프 ‘에너지 휴전’ 발표에 “회담 진행 중”…우크라 공격은 지속  한겨레'에너지 휴전' 놓고 설전..."거래가 아닌 제재할 때"  YTN 사이언스트럼프 ‘에너지 휴전’ 후폭풍 속 침묵하는 푸틴…왜?  경향신문불붙은 세계 ‘경유 전쟁’… 美 제재 풀고 中은 통제  동아일보거래의 기술인가 배신의 외교인가…갈림길에 선...</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>한겨레</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxNSHNsRkxpRGc4OW5TaWk0NTFndFgwM2tpd0xMTWZtaXl2OVpfUHhvc3hNNzNhSDhYT2ZYOFFMUEhzck9hY0RHdC1YUzhzR3ZfMHpydHlUTXlQbko1QzJ4dE96WkFhT2VJS1AycnlIU0xubjlndnZBY3gxbHpoNjZwMmZR?oc=5</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>트럼프 에너지 휴전 선언은 우크라에 '차포 떼라' 압박</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Mon, 12 Oct 2026 23:49:00 GMT</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속 보도)</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>독일 길거리서 로봇이 성추행···SNS 중계 10대들 ‘성적 모욕 혐의’ 수사</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>독일 길거리서 로봇이 성추행···SNS 중계 10대들 ‘성적 모욕 혐의’ 수사  경향신문'아이언맨 색상' 로봇이 여성 성추행…생중계한 범인은 독일 10대들[이런일이]  노컷뉴스獨서 로봇이 10대 여성 성추행…SNS 생중계도  문화일보독일 길거리서 로봇이 성추행…SNS 중계 10대들 수사  연합뉴스한밤중 로봇이 16세女 성...</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>경향신문</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiWkFVX3lxTE1vWFcwSDdLdHdHc1Z5WVBXbjI5em1iU2tpdFllaXN5eG1vdzNoaEt3aGVGME05aXllTGlVS3pYRXpQWTgxZEV0QWwxNkV4RUxOMWNNZjg1c3kyQdIBX0FVX3lxTE1qdFNKaHVxbXl0d1dtZmZtdEZMeU0tMUtNZV91LUlmS05XTFZKVFNxTUIzcWh3NllOY1VDdW54cmFibzdIZk1iMjVVSThyWnZqVGQtamtZSy1BQ19mVW40?oc=5</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>로봇이 길거리서 여성 성추행했다…틱톡 중계한 독일 10대 체포</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>Mon, 12 Oct 2026 23:29:00 GMT</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>연결 이슈 (후속 보도)</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>네팔 홍수로 외국인 관광객 100여명 고립…321명 구조·주민 5명 실종</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>네팔 홍수로 외국인 관광객 100여명 고립…321명 구조·주민 5명 실종  강원도민일보네팔, 또 다시 산사태로 홍수 발생···최소 5명 실종  경향신문네팔 홍수로 외국인 관광객 100여명 고립…헬기 구조에도 발 묶여  뉴시스남동발전, ’네팔 대홍수’ 수색 일시 중단…“재개 여부 추후 결정“  연합뉴스TV네팔 산사태로 강 ...</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>강원도민일보</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE1hRG8yTXNrdU4wUHZhUnFMR3RRRTMxcEtoT1FzTEhyS0RxS0ltVWd4NGxGWWNjU1FlSkcwTm11cnVmZktRX3F1cFBsdTZWWHlCejBTX1B3RW1Ub3lEWHNSdlYwbExWLVU?oc=5</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>네팔 홍수로 외국인 트레킹객 100여명 고립…등산로·교량 유실</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 02:23:10 GMT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>세계/국제</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>트럼프, 아시아 방문 중 김정은과 회담 계획 묻자 "그럴 수도"</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>트럼프, 아시아 방문 중 김정은과 회담 계획 묻자 "그럴 수도"  연합뉴스TV트럼프 "다음 달 김정은 위원장과 만날 수도...흥미진진할 것"  YTN 사이언스[속보]트럼프, 아시아 방문중 김정은과 회담계획 묻자 “그럴 수도”  문화일보다음 달 중국가는 트럼프… 김정은과 회담 계획 묻자 "그럴 수도"  조선일보트럼프, 김정...</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>연합뉴스TV</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMiZ0FVX3lxTE5Zbkt0YjdRTXlYZ0h5UzF0bUNLQjNDMnNORTlTTkcwV3BkejE0WVhiaVVZVERwVmN1bTlFNjNxYnNOSTRjaGpNOUtGeGpVbXJvdHBZNlBPdWJIUlpvRWJudjk5cEJrb28?oc=5</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>Mon, 12 Oct 2026 21:25:00 GMT</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>IT/과학/신상품</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>신규 이슈</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>아이폰 사진 뿌옇게 나온다면…촬영 전 반드시 점검해야 할 것들</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>아이폰 사진 뿌옇게 나온다면…촬영 전 반드시 점검해야 할 것들  디지털투데이</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>디지털투데이</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>https://news.google.com/rss/articles/CBMic0FVX3lxTFBmdTNGVjRhOUNyamdIWWY1SnZha0U2MWhWcEZ4ZGZ3T3g1Sll6SVpwQnljdWozWjViWDY0SXN4el9zV0hFM3A3OHd2ZHdQYXI5RDQwV3IyRlBPWWFOdUFoUno5bFZsOGpvQjR0MXRtaXo2U00?oc=5</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Tue, 13 Oct 2026 05:33:57 GMT</t>
+          <t>https://www.yna.co.kr/view/AKR20261013167300052</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Tue, 13 Oct 2026 17:27:08 +0900</t>
         </is>
       </c>
     </row>
@@ -1022,13 +773,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="51" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1052,6 +807,10 @@
           <t>참고</t>
         </is>
       </c>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2">
@@ -1061,6 +820,10 @@
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1083,6 +846,10 @@
           <t>실시간 마켓 데이터</t>
         </is>
       </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1105,12 +872,20 @@
           <t>실시간 마켓 데이터</t>
         </is>
       </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2">
@@ -1120,6 +895,10 @@
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1142,6 +921,10 @@
           <t>실시간 외환 데이터</t>
         </is>
       </c>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1164,6 +947,10 @@
           <t>실시간 외환 데이터</t>
         </is>
       </c>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1186,6 +973,10 @@
           <t>실시간 외환 데이터</t>
         </is>
       </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1208,12 +999,492 @@
           <t>실시간 외환 데이터</t>
         </is>
       </c>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr"/>
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>상태</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>관련기업/기관</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>기사제목</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>영향/전망</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>언론사</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>요약</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>링크</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>삼양컴텍</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>[신한투자증권] 삼양컴텍: 구미공장 탐방: 증설 끝, 이제 폴란드형 K2</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>신한투자증권</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 868회</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96677</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>현대모비스</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>[한화투자증권] 현대모비스: 불리한 매크로 영향 지속, 구조적 수익성 개선도 지속</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>한화투자증권</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 1,861회</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96676</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>현대글로비스</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>[한화투자증권] 현대글로비스: 고유가로 이익 개선 가시성 둔화, 그러나 증익 방향성 명확</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>한화투자증권</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 1,461회</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96675</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>삼성중공업</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>[DS투자증권] 삼성중공업: 3Q26 Preview: 증익의 시작점</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>DS투자증권</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 2,116회</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96674</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>휴젤</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>[교보증권] 휴젤: 3Q26 Preview: 쉬어가는 한 분기</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>교보증권</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 1,467회</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96673</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>에이피알</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>[교보증권] 에이피알: 환율은 부담이나, 4분기 메인 시즌 기대</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>교보증권</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 2,883회</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96672</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>SK하이닉스</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>[하나증권] SK하이닉스: 컨센서스에 부합</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 6,514회</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96671</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>키움증권</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>[하나증권] 키움증권: 3Q26 Pre - 배당을 바라보며</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 1,478회</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96670</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>한국금융지주</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>[하나증권] 한국금융지주: 3Q26 Pre - 실적 눈높이 조정 구간</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 1,563회</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96669</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>증권사 리서치</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>전문 리포트</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>KT</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>[하나증권] KT: 3Q 프리뷰 - 2027년도 내다본 매수 추천</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>📘 애널리스트 리포트</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>하나증권</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>조회수: 1,581회</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>https://m.stock.naver.com/research/company/96668</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1242,7 +1513,7 @@
     <col width="34" customWidth="1" min="11" max="11"/>
     <col width="65" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="65" customWidth="1" min="14" max="14"/>
+    <col width="64" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1377,11 +1648,11 @@
         </is>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>[환율 전망] 대외 악재는 산더미, 반도체 하나로 딸깍 (KB Think)</t>
         </is>
       </c>
     </row>
@@ -1445,11 +1716,11 @@
         </is>
       </c>
       <c r="M3" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t>최근 특이 뉴스 없음</t>
+          <t>[하나증권] SK하이닉스: 컨센서스에 부합 (하나증권)</t>
         </is>
       </c>
     </row>
@@ -2125,11 +2396,11 @@
         </is>
       </c>
       <c r="M13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N13" s="3" t="inlineStr">
         <is>
-          <t>아이폰 사진 뿌옇게 나온다면…촬영 전 반드시 점검해야 할 것들 (디지털투데이)</t>
+          <t>최근 특이 뉴스 없음</t>
         </is>
       </c>
     </row>

</xml_diff>